<commit_message>
QA dashboard save: Maple Grove Home Health
</commit_message>
<xml_diff>
--- a/qa-data/HomeHealth-Data-QA.xlsx
+++ b/qa-data/HomeHealth-Data-QA.xlsx
@@ -1036,13 +1036,13 @@
         <v>24</v>
       </c>
       <c r="C13" s="1">
-        <v>86</v>
-      </c>
-      <c r="D13">
-        <v>0.865</v>
+        <v>90</v>
+      </c>
+      <c r="D13" s="1">
+        <v>0.9</v>
       </c>
       <c r="E13" s="1">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="F13">
         <v>348.13</v>
@@ -1051,19 +1051,19 @@
         <v>270.08</v>
       </c>
       <c r="H13" s="1">
-        <v>788200</v>
+        <v>800000</v>
       </c>
       <c r="I13" s="1">
-        <v>724120</v>
+        <v>765000</v>
       </c>
       <c r="J13" s="1">
-        <v>64080</v>
+        <v>35000</v>
       </c>
       <c r="K13" s="1">
-        <v>8420</v>
+        <v>8500</v>
       </c>
       <c r="L13" s="1">
-        <v>0.0813</v>
+        <v>0.0438</v>
       </c>
     </row>
     <row r="14" ht="15.5" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -3263,28 +3263,28 @@
         <v>24</v>
       </c>
       <c r="B13" s="1">
-        <v>496</v>
+        <v>474</v>
       </c>
       <c r="C13" s="1">
-        <v>439</v>
+        <v>422</v>
       </c>
       <c r="D13" s="1">
-        <v>0.8851</v>
+        <v>0.8903</v>
       </c>
       <c r="E13" s="1">
-        <v>4521095.99</v>
+        <v>4532895.85</v>
       </c>
       <c r="F13" s="1">
-        <v>4243909.68</v>
+        <v>4047941.68</v>
       </c>
       <c r="G13" s="1">
-        <v>277186.31</v>
+        <v>484954.17</v>
       </c>
       <c r="H13" s="1">
-        <v>0.0613</v>
+        <v>0.107</v>
       </c>
       <c r="I13" s="1">
-        <v>8556.27</v>
+        <v>8539.96</v>
       </c>
     </row>
   </sheetData>
@@ -3350,34 +3350,34 @@
         <v>12</v>
       </c>
       <c r="B2" s="1">
-        <v>86</v>
-      </c>
-      <c r="C2">
-        <v>0.865</v>
+        <v>90</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.9</v>
       </c>
       <c r="D2" s="1">
-        <v>788200</v>
+        <v>800000</v>
       </c>
       <c r="E2" s="1">
-        <v>724120</v>
+        <v>765000</v>
       </c>
       <c r="F2" s="1">
-        <v>64080</v>
+        <v>35000</v>
       </c>
       <c r="G2" s="1">
-        <v>8420</v>
+        <v>8500</v>
       </c>
       <c r="H2" s="1">
-        <v>0.0813</v>
+        <v>0.0438</v>
       </c>
       <c r="I2" s="1">
-        <v>0.0045</v>
+        <v>0.0195</v>
       </c>
       <c r="J2" s="1">
-        <v>8879243.4</v>
+        <v>8891043.4</v>
       </c>
       <c r="K2" s="1">
-        <v>703777.66</v>
+        <v>674697.66</v>
       </c>
     </row>
     <row r="3" ht="15.5" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
QA dashboard save: Riverside Care Center
</commit_message>
<xml_diff>
--- a/qa-data/HomeHealth-Data-QA.xlsx
+++ b/qa-data/HomeHealth-Data-QA.xlsx
@@ -1492,13 +1492,13 @@
         <v>24</v>
       </c>
       <c r="C25" s="1">
-        <v>136</v>
-      </c>
-      <c r="D25">
-        <v>0.902</v>
+        <v>125</v>
+      </c>
+      <c r="D25" s="1">
+        <v>0.91</v>
       </c>
       <c r="E25" s="1">
-        <v>123</v>
+        <v>114</v>
       </c>
       <c r="F25">
         <v>358.62</v>
@@ -1506,20 +1506,20 @@
       <c r="G25">
         <v>280.54</v>
       </c>
-      <c r="H25">
-        <v>1200663</v>
+      <c r="H25" s="1">
+        <v>1250000</v>
       </c>
       <c r="I25" s="1">
-        <v>1182792</v>
+        <v>1100000</v>
       </c>
       <c r="J25" s="1">
-        <v>17871</v>
-      </c>
-      <c r="K25">
-        <v>8697</v>
+        <v>150000</v>
+      </c>
+      <c r="K25" s="1">
+        <v>8800</v>
       </c>
       <c r="L25" s="1">
-        <v>0.0149</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="26" ht="15.5" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -3263,28 +3263,28 @@
         <v>24</v>
       </c>
       <c r="B13" s="1">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="C13" s="1">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D13" s="1">
-        <v>0.8903</v>
+        <v>0.8879</v>
       </c>
       <c r="E13" s="1">
-        <v>4532895.85</v>
+        <v>4570052.67</v>
       </c>
       <c r="F13" s="1">
-        <v>4047941.68</v>
+        <v>4042615.65</v>
       </c>
       <c r="G13" s="1">
-        <v>484954.17</v>
+        <v>527437.02</v>
       </c>
       <c r="H13" s="1">
-        <v>0.107</v>
+        <v>0.1154</v>
       </c>
       <c r="I13" s="1">
-        <v>8539.96</v>
+        <v>8546.76</v>
       </c>
     </row>
   </sheetData>
@@ -3385,34 +3385,34 @@
         <v>25</v>
       </c>
       <c r="B3" s="1">
-        <v>136</v>
-      </c>
-      <c r="C3">
-        <v>0.902</v>
-      </c>
-      <c r="D3">
-        <v>1200663</v>
+        <v>125</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0.91</v>
+      </c>
+      <c r="D3" s="1">
+        <v>1250000</v>
       </c>
       <c r="E3" s="1">
-        <v>1182792</v>
+        <v>1100000</v>
       </c>
       <c r="F3" s="1">
-        <v>17871</v>
-      </c>
-      <c r="G3">
-        <v>8697</v>
+        <v>150000</v>
+      </c>
+      <c r="G3" s="1">
+        <v>8800</v>
       </c>
       <c r="H3" s="1">
-        <v>0.0149</v>
-      </c>
-      <c r="I3">
-        <v>-0.0137</v>
-      </c>
-      <c r="J3">
-        <v>13910058.93</v>
+        <v>0.12</v>
+      </c>
+      <c r="I3" s="1">
+        <v>0.0268</v>
+      </c>
+      <c r="J3" s="1">
+        <v>13959395.93</v>
       </c>
       <c r="K3" s="1">
-        <v>1710940.96</v>
+        <v>1843069.96</v>
       </c>
     </row>
     <row r="4" ht="15.5" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
QA dashboard save: Maple Grove Home Health, Riverside Care Center, Cedar Point Nursing, Willow Creek Rehab
</commit_message>
<xml_diff>
--- a/qa-data/HomeHealth-Data-QA.xlsx
+++ b/qa-data/HomeHealth-Data-QA.xlsx
@@ -1036,13 +1036,13 @@
         <v>24</v>
       </c>
       <c r="C13" s="1">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="D13" s="1">
-        <v>0.9</v>
+        <v>0.865</v>
       </c>
       <c r="E13" s="1">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="F13">
         <v>348.13</v>
@@ -1051,19 +1051,19 @@
         <v>270.08</v>
       </c>
       <c r="H13" s="1">
-        <v>800000</v>
+        <v>787820</v>
       </c>
       <c r="I13" s="1">
-        <v>765000</v>
+        <v>879060</v>
       </c>
       <c r="J13" s="1">
-        <v>35000</v>
+        <v>-91240</v>
       </c>
       <c r="K13" s="1">
-        <v>8500</v>
+        <v>8372</v>
       </c>
       <c r="L13" s="1">
-        <v>0.0438</v>
+        <v>-0.1158</v>
       </c>
     </row>
     <row r="14" ht="15.5" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1492,13 +1492,13 @@
         <v>24</v>
       </c>
       <c r="C25" s="1">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="D25" s="1">
-        <v>0.91</v>
+        <v>0.902</v>
       </c>
       <c r="E25" s="1">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="F25">
         <v>358.62</v>
@@ -1507,19 +1507,19 @@
         <v>280.54</v>
       </c>
       <c r="H25" s="1">
-        <v>1250000</v>
+        <v>1200663</v>
       </c>
       <c r="I25" s="1">
-        <v>1100000</v>
+        <v>1064400</v>
       </c>
       <c r="J25" s="1">
-        <v>150000</v>
+        <v>136263</v>
       </c>
       <c r="K25" s="1">
-        <v>8800</v>
+        <v>8870</v>
       </c>
       <c r="L25" s="1">
-        <v>0.12</v>
+        <v>0.1135</v>
       </c>
     </row>
     <row r="26" ht="15.5" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1948,13 +1948,13 @@
         <v>24</v>
       </c>
       <c r="C37" s="1">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="D37">
         <v>0.836</v>
       </c>
       <c r="E37" s="1">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="F37">
         <v>335.05</v>
@@ -1966,16 +1966,16 @@
         <v>830934</v>
       </c>
       <c r="I37" s="1">
-        <v>845630</v>
+        <v>949572</v>
       </c>
       <c r="J37" s="1">
-        <v>-14696</v>
+        <v>-118638</v>
       </c>
       <c r="K37" s="1">
-        <v>8210</v>
+        <v>8116</v>
       </c>
       <c r="L37" s="1">
-        <v>-0.0177</v>
+        <v>-0.1428</v>
       </c>
     </row>
     <row r="38" ht="15.5" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -2404,13 +2404,13 @@
         <v>24</v>
       </c>
       <c r="C49" s="1">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="D49">
         <v>0.947</v>
       </c>
       <c r="E49" s="1">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="F49">
         <v>374.15</v>
@@ -2422,16 +2422,16 @@
         <v>661116</v>
       </c>
       <c r="I49" s="1">
-        <v>579600</v>
+        <v>814880</v>
       </c>
       <c r="J49" s="1">
-        <v>81516</v>
+        <v>-153764</v>
       </c>
       <c r="K49" s="1">
-        <v>9200</v>
+        <v>9260</v>
       </c>
       <c r="L49" s="1">
-        <v>0.1233</v>
+        <v>-0.2326</v>
       </c>
     </row>
     <row r="50" ht="15.5" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -3263,28 +3263,28 @@
         <v>24</v>
       </c>
       <c r="B13" s="1">
-        <v>473</v>
+        <v>538</v>
       </c>
       <c r="C13" s="1">
-        <v>420</v>
+        <v>476</v>
       </c>
       <c r="D13" s="1">
-        <v>0.8879</v>
+        <v>0.8848</v>
       </c>
       <c r="E13" s="1">
-        <v>4570052.67</v>
+        <v>4520715.99</v>
       </c>
       <c r="F13" s="1">
-        <v>4042615.65</v>
+        <v>4619679.68</v>
       </c>
       <c r="G13" s="1">
-        <v>527437.02</v>
+        <v>-98963.69</v>
       </c>
       <c r="H13" s="1">
-        <v>0.1154</v>
+        <v>-0.0219</v>
       </c>
       <c r="I13" s="1">
-        <v>8546.76</v>
+        <v>8586.77</v>
       </c>
     </row>
   </sheetData>
@@ -3350,34 +3350,34 @@
         <v>12</v>
       </c>
       <c r="B2" s="1">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="C2" s="1">
-        <v>0.9</v>
+        <v>0.865</v>
       </c>
       <c r="D2" s="1">
-        <v>800000</v>
+        <v>787820</v>
       </c>
       <c r="E2" s="1">
-        <v>765000</v>
+        <v>879060</v>
       </c>
       <c r="F2" s="1">
-        <v>35000</v>
+        <v>-91240</v>
       </c>
       <c r="G2" s="1">
-        <v>8500</v>
+        <v>8372</v>
       </c>
       <c r="H2" s="1">
-        <v>0.0438</v>
+        <v>-0.1158</v>
       </c>
       <c r="I2" s="1">
-        <v>0.0195</v>
+        <v>0.004</v>
       </c>
       <c r="J2" s="1">
-        <v>8891043.4</v>
+        <v>8878863.4</v>
       </c>
       <c r="K2" s="1">
-        <v>674697.66</v>
+        <v>548457.66</v>
       </c>
     </row>
     <row r="3" ht="15.5" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -3385,34 +3385,34 @@
         <v>25</v>
       </c>
       <c r="B3" s="1">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C3" s="1">
-        <v>0.91</v>
+        <v>0.902</v>
       </c>
       <c r="D3" s="1">
-        <v>1250000</v>
+        <v>1200663</v>
       </c>
       <c r="E3" s="1">
-        <v>1100000</v>
+        <v>1064400</v>
       </c>
       <c r="F3" s="1">
-        <v>150000</v>
+        <v>136263</v>
       </c>
       <c r="G3" s="1">
-        <v>8800</v>
+        <v>8870</v>
       </c>
       <c r="H3" s="1">
-        <v>0.12</v>
+        <v>0.1135</v>
       </c>
       <c r="I3" s="1">
-        <v>0.0268</v>
+        <v>-0.0137</v>
       </c>
       <c r="J3" s="1">
-        <v>13959395.93</v>
+        <v>13910058.93</v>
       </c>
       <c r="K3" s="1">
-        <v>1843069.96</v>
+        <v>1829332.96</v>
       </c>
     </row>
     <row r="4" ht="15.5" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -3420,7 +3420,7 @@
         <v>26</v>
       </c>
       <c r="B4" s="1">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="C4">
         <v>0.836</v>
@@ -3429,16 +3429,16 @@
         <v>830934</v>
       </c>
       <c r="E4" s="1">
-        <v>845630</v>
+        <v>949572</v>
       </c>
       <c r="F4" s="1">
-        <v>-14696</v>
+        <v>-118638</v>
       </c>
       <c r="G4" s="1">
-        <v>8210</v>
+        <v>8116</v>
       </c>
       <c r="H4" s="1">
-        <v>-0.0177</v>
+        <v>-0.1428</v>
       </c>
       <c r="I4">
         <v>0.0004</v>
@@ -3447,7 +3447,7 @@
         <v>9411596.38</v>
       </c>
       <c r="K4" s="1">
-        <v>286200.36</v>
+        <v>182258.36</v>
       </c>
     </row>
     <row r="5" ht="15.5" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -3455,7 +3455,7 @@
         <v>27</v>
       </c>
       <c r="B5" s="1">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="C5">
         <v>0.947</v>
@@ -3464,16 +3464,16 @@
         <v>661116</v>
       </c>
       <c r="E5" s="1">
-        <v>579600</v>
+        <v>814880</v>
       </c>
       <c r="F5" s="1">
-        <v>81516</v>
+        <v>-153764</v>
       </c>
       <c r="G5" s="1">
-        <v>9200</v>
+        <v>9260</v>
       </c>
       <c r="H5" s="1">
-        <v>0.1233</v>
+        <v>-0.2326</v>
       </c>
       <c r="I5">
         <v>0.0012</v>
@@ -3482,7 +3482,7 @@
         <v>7429588.17</v>
       </c>
       <c r="K5" s="1">
-        <v>989032.02</v>
+        <v>753752.02</v>
       </c>
     </row>
     <row r="6" ht="15.5" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>